<commit_message>
Final Latihan ERD dan Query
</commit_message>
<xml_diff>
--- a/Normalisasi_SalesDB_Ilham.xlsx
+++ b/Normalisasi_SalesDB_Ilham.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\hp\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FAB41B93-357B-40EC-A563-CEA3894CD1FD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BF53BAC4-0F12-4428-98E0-07C1ED8F6499}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Petunjuk" sheetId="1" r:id="rId1"/>
@@ -18,7 +18,9 @@
     <sheet name="2_1NF" sheetId="3" r:id="rId3"/>
     <sheet name="3_2NF" sheetId="4" r:id="rId4"/>
     <sheet name="4_3NF" sheetId="5" r:id="rId5"/>
-    <sheet name="Sheet1" sheetId="6" r:id="rId6"/>
+    <sheet name="Query" sheetId="9" r:id="rId6"/>
+    <sheet name="Diagram" sheetId="8" r:id="rId7"/>
+    <sheet name="Buat pisah pisahin" sheetId="6" r:id="rId8"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -143,7 +145,7 @@
     <author>Trainer</author>
   </authors>
   <commentList>
-    <comment ref="C15" authorId="0" shapeId="0" xr:uid="{9A8263C8-9E30-4D69-9FD5-7E8767182EE1}">
+    <comment ref="D41" authorId="0" shapeId="0" xr:uid="{9A8263C8-9E30-4D69-9FD5-7E8767182EE1}">
       <text>
         <r>
           <rPr>
@@ -157,7 +159,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="C16" authorId="0" shapeId="0" xr:uid="{846807AA-BD49-44FC-A1A1-96DCB7AE3F24}">
+    <comment ref="D42" authorId="0" shapeId="0" xr:uid="{846807AA-BD49-44FC-A1A1-96DCB7AE3F24}">
       <text>
         <r>
           <rPr>
@@ -256,7 +258,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="755" uniqueCount="144">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="880" uniqueCount="253">
   <si>
     <t>Latihan Normalisasi SalesDB — dari data faktur (UNF) sampai 3NF</t>
   </si>
@@ -713,12 +715,6 @@
     <t>Kode Produk (PK)</t>
   </si>
   <si>
-    <t xml:space="preserve">No Faktur (PK,FK) </t>
-  </si>
-  <si>
-    <t>Kode Produk (PK, FK)</t>
-  </si>
-  <si>
     <t>Kode Kategori (FK)</t>
   </si>
   <si>
@@ -729,6 +725,339 @@
   </si>
   <si>
     <t>NO FAKTUR -&gt; KODE PELANGGAN,</t>
+  </si>
+  <si>
+    <t>No faktur (PK,FK)</t>
+  </si>
+  <si>
+    <t>Kode Produk (PK,FK)</t>
+  </si>
+  <si>
+    <t>Orders</t>
+  </si>
+  <si>
+    <t>Customer</t>
+  </si>
+  <si>
+    <t>USE master</t>
+  </si>
+  <si>
+    <t>GO</t>
+  </si>
+  <si>
+    <t xml:space="preserve">IF DB_ID ('SalesDB') IS NOT NULL </t>
+  </si>
+  <si>
+    <t>BEGIN</t>
+  </si>
+  <si>
+    <t>DROP DATABASE SalesDB;</t>
+  </si>
+  <si>
+    <t>END</t>
+  </si>
+  <si>
+    <t>CREATE DATABASE SalesDB</t>
+  </si>
+  <si>
+    <t>USE SalesDB</t>
+  </si>
+  <si>
+    <t>CREATE TABLE Customer (</t>
+  </si>
+  <si>
+    <t>CustomerID uniqueidentifier not null PRIMARY KEY Default NEWID(),</t>
+  </si>
+  <si>
+    <t>CustomerName Nvarchar(50) not null,</t>
+  </si>
+  <si>
+    <t>Email Nvarchar(50) not null,</t>
+  </si>
+  <si>
+    <t>City Nvarchar(50) not null</t>
+  </si>
+  <si>
+    <t>)</t>
+  </si>
+  <si>
+    <t>CREATE UNIQUE NONCLUSTERED INDEX UQ_Customer_Email</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ON dbo.Customer (Email) </t>
+  </si>
+  <si>
+    <t xml:space="preserve">WHERE Email IS NOT NULL; </t>
+  </si>
+  <si>
+    <t>CREATE TABLE Orders(</t>
+  </si>
+  <si>
+    <t>OrderID uniqueidentifier not null PRIMARY KEY Default NEWID(),</t>
+  </si>
+  <si>
+    <t>OrderDate datetime2 not null Default GETDATE(),</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CustomerID uniqueidentifier NOT NULL, </t>
+  </si>
+  <si>
+    <t>CREATE TABLE Category(</t>
+  </si>
+  <si>
+    <t>CategoryID int not null PRIMARY KEY IDENTITY(1,1),</t>
+  </si>
+  <si>
+    <t>CategoryName NVARCHAR(50) not null,</t>
+  </si>
+  <si>
+    <t>SubCategoryID int,</t>
+  </si>
+  <si>
+    <t>CREATE TABLE Products(</t>
+  </si>
+  <si>
+    <t>ProductID int not null PRIMARY KEY IDENTITY(1,1),</t>
+  </si>
+  <si>
+    <t>ProductName NVARCHAR(50) not null,</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Price decimal(12,2) NOT NULL, </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Stock int NOT NULL, </t>
+  </si>
+  <si>
+    <t>CategoryID int not null,</t>
+  </si>
+  <si>
+    <t>CREATE TABLE OrderDetail(</t>
+  </si>
+  <si>
+    <t>OrderID uniqueidentifier not null Default NEWID(),</t>
+  </si>
+  <si>
+    <t>ProductID int not null,</t>
+  </si>
+  <si>
+    <t>Quantity int check(quantity &gt; 0),</t>
+  </si>
+  <si>
+    <t>UnitPrice decimal(12,2)</t>
+  </si>
+  <si>
+    <t>PRIMARY KEY (OrderID, ProductID),</t>
+  </si>
+  <si>
+    <t>ALTER TABLE Customer</t>
+  </si>
+  <si>
+    <t>ADD CONSTRAINT FK_Customer</t>
+  </si>
+  <si>
+    <t>foreign key (CustomerID) references Customer(CustomerID)</t>
+  </si>
+  <si>
+    <t>ON DELETE NO ACTION</t>
+  </si>
+  <si>
+    <t>ON UPDATE NO ACTION</t>
+  </si>
+  <si>
+    <t>ALTER TABLE Category</t>
+  </si>
+  <si>
+    <t>ADD CONSTRAINT FK_Category</t>
+  </si>
+  <si>
+    <t>Foreign key (SubCategoryID) references Category(CategoryID)</t>
+  </si>
+  <si>
+    <t>ALTER TABLE Products</t>
+  </si>
+  <si>
+    <t>ADD CONSTRAINT FK_Product</t>
+  </si>
+  <si>
+    <t>foreign key (CategoryID) references Category(CategoryID)</t>
+  </si>
+  <si>
+    <t>ALTER TABLE OrderDetail</t>
+  </si>
+  <si>
+    <t>ADD CONSTRAINT FK_OrderDetail</t>
+  </si>
+  <si>
+    <t>foreign key (OrderID) references Orders(OrderID),</t>
+  </si>
+  <si>
+    <t>foreign key (ProductID) references Products(ProductID)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">INSERT INTO Category VALUES </t>
+  </si>
+  <si>
+    <t>('Elektronik', NULL),</t>
+  </si>
+  <si>
+    <t>('Alat Tulis', NULL),</t>
+  </si>
+  <si>
+    <t>('Aksesoris Komputer', NULL)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">INSERT INTO Products VALUES </t>
+  </si>
+  <si>
+    <t>('Monitor 24 Inci', '1850000', 50, 1),</t>
+  </si>
+  <si>
+    <t>('Mouse Wireless', '150000', 25, 3),</t>
+  </si>
+  <si>
+    <t>('Keyboard Mekanik', '750000',30, 3),</t>
+  </si>
+  <si>
+    <t>('Headset USB', '150000', 40,1),</t>
+  </si>
+  <si>
+    <t>('Buku Catatan A5', '350000',15, 2),</t>
+  </si>
+  <si>
+    <t>('Pulpen Gel (isi 12)', '25000',100, 1)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">INSERT INTO Customer VALUES </t>
+  </si>
+  <si>
+    <t>(NEWID(), 'Andi Wijaya',</t>
+  </si>
+  <si>
+    <t>'andi@mail.com','Surabaya'),</t>
+  </si>
+  <si>
+    <t>(NEWID(),'Budi Santoso',</t>
+  </si>
+  <si>
+    <t>'budi@mail.com','Jakarta'),</t>
+  </si>
+  <si>
+    <t>(NEWID(), 'Siti Aminah',</t>
+  </si>
+  <si>
+    <t>'siti@mail.com','Bandung')</t>
+  </si>
+  <si>
+    <t>INSERT INTO Orders VALUES</t>
+  </si>
+  <si>
+    <t>(NEWID(), '2026-09-01',</t>
+  </si>
+  <si>
+    <t>'C04710A5-EE2A-4253-8A94-6BDF2B562BC5'),</t>
+  </si>
+  <si>
+    <t>(NEWID(), '2026-09-10',</t>
+  </si>
+  <si>
+    <t>'465454AA-F03C-4216-8A1D-BADFF5CC1280'),</t>
+  </si>
+  <si>
+    <t>(NEWID(), '2026-09-12',</t>
+  </si>
+  <si>
+    <t>'592A6119-7DBE-4A6C-90F5-EE9380D13EFF'),</t>
+  </si>
+  <si>
+    <t>(NEWID(), '2026-09-15',</t>
+  </si>
+  <si>
+    <t>(NEWID(), '2026-09-18',</t>
+  </si>
+  <si>
+    <t>(NEWID(), '2026-09-20',</t>
+  </si>
+  <si>
+    <t>'592A6119-7DBE-4A6C-90F5-EE9380D13EFF');</t>
+  </si>
+  <si>
+    <t>INSERT INTO OrderDetail VALUES</t>
+  </si>
+  <si>
+    <t>('BCD7E79E-E4A2-4F56-99D4-4A8D21515417',1,1,'1850000'),</t>
+  </si>
+  <si>
+    <t>('BCD7E79E-E4A2-4F56-99D4-4A8D21515417',2,2,'300000'),</t>
+  </si>
+  <si>
+    <t>('489180ED-3847-4F77-9D31-35A9FB508536',3,1,'750000'),</t>
+  </si>
+  <si>
+    <t>('489180ED-3847-4F77-9D31-35A9FB508536',2,1,'150000'),</t>
+  </si>
+  <si>
+    <t>('51A180C4-60A2-47B5-8804-44C151ACCEBF',4,3,'1050000'),</t>
+  </si>
+  <si>
+    <t>('FF9D33E8-B7BF-4777-929E-7778022DEADB',5,10,'250000'),</t>
+  </si>
+  <si>
+    <t>('FF9D33E8-B7BF-4777-929E-7778022DEADB',6,2,'96000'),</t>
+  </si>
+  <si>
+    <t>('5C361F32-EFAE-418B-8C4D-4B959E3215B8',4,1,'375000'),</t>
+  </si>
+  <si>
+    <t>('5C361F32-EFAE-418B-8C4D-4B959E3215B8',5,5,'125000'),</t>
+  </si>
+  <si>
+    <t>('5C361F32-EFAE-418B-8C4D-4B959E3215B8',6,1,'48000'),</t>
+  </si>
+  <si>
+    <t>('7F55CD5C-6C32-4DC9-9533-88CBCDD7D590',1,2,'3700000'),</t>
+  </si>
+  <si>
+    <t>('7F55CD5C-6C32-4DC9-9533-88CBCDD7D590',3,1,'1850000')</t>
+  </si>
+  <si>
+    <t>SELECT * FROM Customer</t>
+  </si>
+  <si>
+    <t>SELECT * FROM Orders</t>
+  </si>
+  <si>
+    <t>SELECT * FROM Category</t>
+  </si>
+  <si>
+    <t>SELECT * FROM Products</t>
+  </si>
+  <si>
+    <t>SELECT * FROM OrderDetail</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SELECT CustomerName, Email, City, OrderDate, ProductName, CategoryName, Price, Quantity, UnitPrice FROM Customer </t>
+  </si>
+  <si>
+    <t>JOIN Orders ON Orders.CustomerID = Customer.CustomerID</t>
+  </si>
+  <si>
+    <t>JOIN OrderDetail ON OrderDetail.OrderID = Orders.OrderID</t>
+  </si>
+  <si>
+    <t>JOIN Products ON Products.ProductID = OrderDetail.ProductID</t>
+  </si>
+  <si>
+    <t>JOIN Category ON Category.CategoryID = Products.CategoryID</t>
+  </si>
+  <si>
+    <t>Category</t>
+  </si>
+  <si>
+    <t>OrderDetail</t>
+  </si>
+  <si>
+    <t>Product</t>
   </si>
 </sst>
 </file>
@@ -891,7 +1220,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="27">
+  <cellXfs count="28">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -930,9 +1259,6 @@
     <xf numFmtId="3" fontId="11" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
@@ -943,6 +1269,12 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="9" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -959,6 +1291,61 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>439616</xdr:colOff>
+      <xdr:row>1</xdr:row>
+      <xdr:rowOff>183173</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>16</xdr:col>
+      <xdr:colOff>546589</xdr:colOff>
+      <xdr:row>29</xdr:row>
+      <xdr:rowOff>150935</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="3" name="Picture 2">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{AF7867B2-3073-D93D-ACCF-20E4BD986C6E}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1">
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="439616" y="375505"/>
+          <a:ext cx="9925050" cy="5353050"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1692,93 +2079,93 @@
       </c>
     </row>
     <row r="13" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="B13" s="22" t="s">
+      <c r="B13" s="26" t="s">
         <v>100</v>
       </c>
-      <c r="C13" s="22"/>
-      <c r="D13" s="22"/>
-      <c r="E13" s="22"/>
+      <c r="C13" s="26"/>
+      <c r="D13" s="26"/>
+      <c r="E13" s="26"/>
     </row>
     <row r="14" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A14">
         <v>1</v>
       </c>
-      <c r="B14" s="22" t="s">
+      <c r="B14" s="26" t="s">
         <v>102</v>
       </c>
-      <c r="C14" s="22"/>
-      <c r="D14" s="22"/>
-      <c r="E14" s="22"/>
-      <c r="F14" s="22"/>
-      <c r="G14" s="22"/>
+      <c r="C14" s="26"/>
+      <c r="D14" s="26"/>
+      <c r="E14" s="26"/>
+      <c r="F14" s="26"/>
+      <c r="G14" s="26"/>
     </row>
     <row r="15" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A15">
         <v>2</v>
       </c>
-      <c r="B15" s="22" t="s">
+      <c r="B15" s="26" t="s">
         <v>101</v>
       </c>
-      <c r="C15" s="22"/>
-      <c r="D15" s="22"/>
-      <c r="E15" s="22"/>
-      <c r="F15" s="22"/>
-      <c r="G15" s="22"/>
+      <c r="C15" s="26"/>
+      <c r="D15" s="26"/>
+      <c r="E15" s="26"/>
+      <c r="F15" s="26"/>
+      <c r="G15" s="26"/>
     </row>
     <row r="16" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A16">
         <v>3</v>
       </c>
-      <c r="B16" s="22" t="s">
+      <c r="B16" s="26" t="s">
         <v>105</v>
       </c>
-      <c r="C16" s="22"/>
-      <c r="D16" s="22"/>
-      <c r="E16" s="22"/>
-      <c r="F16" s="22"/>
-      <c r="G16" s="22"/>
+      <c r="C16" s="26"/>
+      <c r="D16" s="26"/>
+      <c r="E16" s="26"/>
+      <c r="F16" s="26"/>
+      <c r="G16" s="26"/>
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A17">
         <v>4</v>
       </c>
-      <c r="B17" s="22" t="s">
+      <c r="B17" s="26" t="s">
         <v>103</v>
       </c>
-      <c r="C17" s="22"/>
-      <c r="D17" s="22"/>
-      <c r="E17" s="22"/>
-      <c r="F17" s="22"/>
-      <c r="G17" s="22"/>
+      <c r="C17" s="26"/>
+      <c r="D17" s="26"/>
+      <c r="E17" s="26"/>
+      <c r="F17" s="26"/>
+      <c r="G17" s="26"/>
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A18">
         <v>5</v>
       </c>
-      <c r="B18" s="22" t="s">
+      <c r="B18" s="26" t="s">
         <v>104</v>
       </c>
-      <c r="C18" s="22"/>
-      <c r="D18" s="22"/>
-      <c r="E18" s="22"/>
-      <c r="F18" s="22"/>
-      <c r="G18" s="22"/>
+      <c r="C18" s="26"/>
+      <c r="D18" s="26"/>
+      <c r="E18" s="26"/>
+      <c r="F18" s="26"/>
+      <c r="G18" s="26"/>
     </row>
     <row r="19" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="B19" s="22"/>
-      <c r="C19" s="22"/>
-      <c r="D19" s="22"/>
-      <c r="E19" s="22"/>
-      <c r="F19" s="22"/>
-      <c r="G19" s="22"/>
+      <c r="B19" s="26"/>
+      <c r="C19" s="26"/>
+      <c r="D19" s="26"/>
+      <c r="E19" s="26"/>
+      <c r="F19" s="26"/>
+      <c r="G19" s="26"/>
     </row>
     <row r="20" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="B20" s="22"/>
-      <c r="C20" s="22"/>
-      <c r="D20" s="22"/>
-      <c r="E20" s="22"/>
-      <c r="F20" s="22"/>
-      <c r="G20" s="22"/>
+      <c r="B20" s="26"/>
+      <c r="C20" s="26"/>
+      <c r="D20" s="26"/>
+      <c r="E20" s="26"/>
+      <c r="F20" s="26"/>
+      <c r="G20" s="26"/>
     </row>
   </sheetData>
   <mergeCells count="8">
@@ -1912,7 +2299,7 @@
       </c>
     </row>
     <row r="12" spans="1:13" ht="28.5" x14ac:dyDescent="0.25">
-      <c r="A12" s="24" t="s">
+      <c r="A12" s="23" t="s">
         <v>35</v>
       </c>
       <c r="B12" s="13">
@@ -1930,7 +2317,7 @@
       <c r="F12" s="12" t="s">
         <v>39</v>
       </c>
-      <c r="G12" s="24" t="s">
+      <c r="G12" s="23" t="s">
         <v>108</v>
       </c>
       <c r="H12" s="12" t="s">
@@ -1953,7 +2340,7 @@
       </c>
     </row>
     <row r="13" spans="1:13" ht="28.5" x14ac:dyDescent="0.25">
-      <c r="A13" s="24" t="s">
+      <c r="A13" s="23" t="s">
         <v>35</v>
       </c>
       <c r="B13" s="13">
@@ -1971,7 +2358,7 @@
       <c r="F13" s="12" t="s">
         <v>39</v>
       </c>
-      <c r="G13" s="24" t="s">
+      <c r="G13" s="23" t="s">
         <v>109</v>
       </c>
       <c r="H13" s="12" t="s">
@@ -1994,7 +2381,7 @@
       </c>
     </row>
     <row r="14" spans="1:13" ht="28.5" x14ac:dyDescent="0.25">
-      <c r="A14" s="24" t="s">
+      <c r="A14" s="23" t="s">
         <v>46</v>
       </c>
       <c r="B14" s="13">
@@ -2012,7 +2399,7 @@
       <c r="F14" s="12" t="s">
         <v>50</v>
       </c>
-      <c r="G14" s="24" t="s">
+      <c r="G14" s="23" t="s">
         <v>115</v>
       </c>
       <c r="H14" s="12" t="s">
@@ -2035,7 +2422,7 @@
       </c>
     </row>
     <row r="15" spans="1:13" ht="28.5" x14ac:dyDescent="0.25">
-      <c r="A15" s="24" t="s">
+      <c r="A15" s="23" t="s">
         <v>46</v>
       </c>
       <c r="B15" s="13">
@@ -2053,7 +2440,7 @@
       <c r="F15" s="12" t="s">
         <v>50</v>
       </c>
-      <c r="G15" s="24" t="s">
+      <c r="G15" s="23" t="s">
         <v>109</v>
       </c>
       <c r="H15" s="12" t="s">
@@ -2076,7 +2463,7 @@
       </c>
     </row>
     <row r="16" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A16" s="24" t="s">
+      <c r="A16" s="23" t="s">
         <v>57</v>
       </c>
       <c r="B16" s="13">
@@ -2094,7 +2481,7 @@
       <c r="F16" s="12" t="s">
         <v>61</v>
       </c>
-      <c r="G16" s="24" t="s">
+      <c r="G16" s="23" t="s">
         <v>62</v>
       </c>
       <c r="H16" s="12" t="s">
@@ -2117,7 +2504,7 @@
       </c>
     </row>
     <row r="17" spans="1:13" ht="28.5" x14ac:dyDescent="0.25">
-      <c r="A17" s="24" t="s">
+      <c r="A17" s="23" t="s">
         <v>68</v>
       </c>
       <c r="B17" s="13">
@@ -2135,7 +2522,7 @@
       <c r="F17" s="12" t="s">
         <v>39</v>
       </c>
-      <c r="G17" s="24" t="s">
+      <c r="G17" s="23" t="s">
         <v>116</v>
       </c>
       <c r="H17" s="12" t="s">
@@ -2158,7 +2545,7 @@
       </c>
     </row>
     <row r="18" spans="1:13" ht="28.5" x14ac:dyDescent="0.25">
-      <c r="A18" s="24" t="s">
+      <c r="A18" s="23" t="s">
         <v>68</v>
       </c>
       <c r="B18" s="13">
@@ -2176,7 +2563,7 @@
       <c r="F18" s="12" t="s">
         <v>39</v>
       </c>
-      <c r="G18" s="24" t="s">
+      <c r="G18" s="23" t="s">
         <v>120</v>
       </c>
       <c r="H18" s="12" t="s">
@@ -2199,7 +2586,7 @@
       </c>
     </row>
     <row r="19" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A19" s="24" t="s">
+      <c r="A19" s="23" t="s">
         <v>75</v>
       </c>
       <c r="B19" s="13">
@@ -2217,7 +2604,7 @@
       <c r="F19" s="12" t="s">
         <v>50</v>
       </c>
-      <c r="G19" s="24" t="s">
+      <c r="G19" s="23" t="s">
         <v>62</v>
       </c>
       <c r="H19" s="12" t="s">
@@ -2240,7 +2627,7 @@
       </c>
     </row>
     <row r="20" spans="1:13" ht="28.5" x14ac:dyDescent="0.25">
-      <c r="A20" s="24" t="s">
+      <c r="A20" s="23" t="s">
         <v>75</v>
       </c>
       <c r="B20" s="13">
@@ -2258,7 +2645,7 @@
       <c r="F20" s="12" t="s">
         <v>50</v>
       </c>
-      <c r="G20" s="24" t="s">
+      <c r="G20" s="23" t="s">
         <v>122</v>
       </c>
       <c r="H20" s="12" t="s">
@@ -2281,7 +2668,7 @@
       </c>
     </row>
     <row r="21" spans="1:13" ht="28.5" x14ac:dyDescent="0.25">
-      <c r="A21" s="24" t="s">
+      <c r="A21" s="23" t="s">
         <v>75</v>
       </c>
       <c r="B21" s="13">
@@ -2299,7 +2686,7 @@
       <c r="F21" s="12" t="s">
         <v>50</v>
       </c>
-      <c r="G21" s="24" t="s">
+      <c r="G21" s="23" t="s">
         <v>120</v>
       </c>
       <c r="H21" s="12" t="s">
@@ -2322,7 +2709,7 @@
       </c>
     </row>
     <row r="22" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A22" s="24" t="s">
+      <c r="A22" s="23" t="s">
         <v>82</v>
       </c>
       <c r="B22" s="13">
@@ -2340,7 +2727,7 @@
       <c r="F22" s="12" t="s">
         <v>61</v>
       </c>
-      <c r="G22" s="24" t="s">
+      <c r="G22" s="23" t="s">
         <v>108</v>
       </c>
       <c r="H22" s="12" t="s">
@@ -2363,7 +2750,7 @@
       </c>
     </row>
     <row r="23" spans="1:13" ht="28.5" x14ac:dyDescent="0.25">
-      <c r="A23" s="24" t="s">
+      <c r="A23" s="23" t="s">
         <v>82</v>
       </c>
       <c r="B23" s="13">
@@ -2381,7 +2768,7 @@
       <c r="F23" s="12" t="s">
         <v>61</v>
       </c>
-      <c r="G23" s="24" t="s">
+      <c r="G23" s="23" t="s">
         <v>126</v>
       </c>
       <c r="H23" s="12" t="s">
@@ -2423,6 +2810,7 @@
     <col min="4" max="4" width="21.7109375" customWidth="1"/>
     <col min="5" max="5" width="28.28515625" customWidth="1"/>
     <col min="6" max="6" width="14.85546875" customWidth="1"/>
+    <col min="7" max="7" width="11.28515625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:7" ht="16.5" x14ac:dyDescent="0.25">
@@ -2502,7 +2890,7 @@
       </c>
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A15" s="24" t="s">
+      <c r="A15" s="23" t="s">
         <v>35</v>
       </c>
       <c r="B15" s="13">
@@ -2525,7 +2913,7 @@
       </c>
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A16" s="24" t="s">
+      <c r="A16" s="23" t="s">
         <v>35</v>
       </c>
       <c r="B16" s="13">
@@ -2548,7 +2936,7 @@
       </c>
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A17" s="24" t="s">
+      <c r="A17" s="23" t="s">
         <v>46</v>
       </c>
       <c r="B17" s="13">
@@ -2571,7 +2959,7 @@
       </c>
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A18" s="24" t="s">
+      <c r="A18" s="23" t="s">
         <v>46</v>
       </c>
       <c r="B18" s="13">
@@ -2594,7 +2982,7 @@
       </c>
     </row>
     <row r="19" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A19" s="24" t="s">
+      <c r="A19" s="23" t="s">
         <v>57</v>
       </c>
       <c r="B19" s="13">
@@ -2617,7 +3005,7 @@
       </c>
     </row>
     <row r="20" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A20" s="24" t="s">
+      <c r="A20" s="23" t="s">
         <v>68</v>
       </c>
       <c r="B20" s="13">
@@ -2640,7 +3028,7 @@
       </c>
     </row>
     <row r="21" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A21" s="24" t="s">
+      <c r="A21" s="23" t="s">
         <v>68</v>
       </c>
       <c r="B21" s="13">
@@ -2663,7 +3051,7 @@
       </c>
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A22" s="24" t="s">
+      <c r="A22" s="23" t="s">
         <v>75</v>
       </c>
       <c r="B22" s="13">
@@ -2686,7 +3074,7 @@
       </c>
     </row>
     <row r="23" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A23" s="24" t="s">
+      <c r="A23" s="23" t="s">
         <v>75</v>
       </c>
       <c r="B23" s="13">
@@ -2709,7 +3097,7 @@
       </c>
     </row>
     <row r="24" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A24" s="24" t="s">
+      <c r="A24" s="23" t="s">
         <v>75</v>
       </c>
       <c r="B24" s="13">
@@ -2732,7 +3120,7 @@
       </c>
     </row>
     <row r="25" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A25" s="24" t="s">
+      <c r="A25" s="23" t="s">
         <v>82</v>
       </c>
       <c r="B25" s="13">
@@ -2755,7 +3143,7 @@
       </c>
     </row>
     <row r="26" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A26" s="24" t="s">
+      <c r="A26" s="23" t="s">
         <v>82</v>
       </c>
       <c r="B26" s="13">
@@ -2792,7 +3180,7 @@
       </c>
     </row>
     <row r="32" spans="1:7" ht="28.5" x14ac:dyDescent="0.25">
-      <c r="A32" s="24" t="s">
+      <c r="A32" s="23" t="s">
         <v>108</v>
       </c>
       <c r="B32" s="12" t="s">
@@ -2806,7 +3194,7 @@
       </c>
     </row>
     <row r="33" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A33" s="24" t="s">
+      <c r="A33" s="23" t="s">
         <v>109</v>
       </c>
       <c r="B33" s="12" t="s">
@@ -2820,7 +3208,7 @@
       </c>
     </row>
     <row r="34" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A34" s="24" t="s">
+      <c r="A34" s="23" t="s">
         <v>115</v>
       </c>
       <c r="B34" s="12" t="s">
@@ -2834,7 +3222,7 @@
       </c>
     </row>
     <row r="35" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A35" s="24" t="s">
+      <c r="A35" s="23" t="s">
         <v>109</v>
       </c>
       <c r="B35" s="12" t="s">
@@ -2848,7 +3236,7 @@
       </c>
     </row>
     <row r="36" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A36" s="24" t="s">
+      <c r="A36" s="23" t="s">
         <v>62</v>
       </c>
       <c r="B36" s="12" t="s">
@@ -2862,7 +3250,7 @@
       </c>
     </row>
     <row r="37" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A37" s="24" t="s">
+      <c r="A37" s="23" t="s">
         <v>116</v>
       </c>
       <c r="B37" s="12" t="s">
@@ -2876,7 +3264,7 @@
       </c>
     </row>
     <row r="38" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A38" s="24" t="s">
+      <c r="A38" s="23" t="s">
         <v>120</v>
       </c>
       <c r="B38" s="12" t="s">
@@ -2890,7 +3278,7 @@
       </c>
     </row>
     <row r="39" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A39" s="24" t="s">
+      <c r="A39" s="23" t="s">
         <v>62</v>
       </c>
       <c r="B39" s="12" t="s">
@@ -2904,7 +3292,7 @@
       </c>
     </row>
     <row r="40" spans="1:4" ht="28.5" x14ac:dyDescent="0.25">
-      <c r="A40" s="24" t="s">
+      <c r="A40" s="23" t="s">
         <v>122</v>
       </c>
       <c r="B40" s="12" t="s">
@@ -2918,7 +3306,7 @@
       </c>
     </row>
     <row r="41" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A41" s="24" t="s">
+      <c r="A41" s="23" t="s">
         <v>120</v>
       </c>
       <c r="B41" s="12" t="s">
@@ -2932,7 +3320,7 @@
       </c>
     </row>
     <row r="42" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A42" s="24" t="s">
+      <c r="A42" s="23" t="s">
         <v>108</v>
       </c>
       <c r="B42" s="12" t="s">
@@ -2946,7 +3334,7 @@
       </c>
     </row>
     <row r="43" spans="1:4" ht="28.5" x14ac:dyDescent="0.25">
-      <c r="A43" s="24" t="s">
+      <c r="A43" s="23" t="s">
         <v>126</v>
       </c>
       <c r="B43" s="12" t="s">
@@ -2974,10 +3362,10 @@
       </c>
     </row>
     <row r="48" spans="1:4" ht="28.5" x14ac:dyDescent="0.25">
-      <c r="A48" s="24" t="s">
+      <c r="A48" s="23" t="s">
         <v>35</v>
       </c>
-      <c r="B48" s="24" t="s">
+      <c r="B48" s="23" t="s">
         <v>108</v>
       </c>
       <c r="C48" s="19">
@@ -2988,10 +3376,10 @@
       </c>
     </row>
     <row r="49" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A49" s="24" t="s">
+      <c r="A49" s="23" t="s">
         <v>35</v>
       </c>
-      <c r="B49" s="24" t="s">
+      <c r="B49" s="23" t="s">
         <v>109</v>
       </c>
       <c r="C49" s="12">
@@ -3002,10 +3390,10 @@
       </c>
     </row>
     <row r="50" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A50" s="24" t="s">
+      <c r="A50" s="23" t="s">
         <v>46</v>
       </c>
-      <c r="B50" s="24" t="s">
+      <c r="B50" s="23" t="s">
         <v>115</v>
       </c>
       <c r="C50" s="12">
@@ -3016,10 +3404,10 @@
       </c>
     </row>
     <row r="51" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A51" s="24" t="s">
+      <c r="A51" s="23" t="s">
         <v>46</v>
       </c>
-      <c r="B51" s="24" t="s">
+      <c r="B51" s="23" t="s">
         <v>109</v>
       </c>
       <c r="C51" s="12">
@@ -3030,10 +3418,10 @@
       </c>
     </row>
     <row r="52" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A52" s="24" t="s">
+      <c r="A52" s="23" t="s">
         <v>57</v>
       </c>
-      <c r="B52" s="24" t="s">
+      <c r="B52" s="23" t="s">
         <v>62</v>
       </c>
       <c r="C52" s="12">
@@ -3044,10 +3432,10 @@
       </c>
     </row>
     <row r="53" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A53" s="24" t="s">
+      <c r="A53" s="23" t="s">
         <v>68</v>
       </c>
-      <c r="B53" s="24" t="s">
+      <c r="B53" s="23" t="s">
         <v>116</v>
       </c>
       <c r="C53" s="12">
@@ -3058,10 +3446,10 @@
       </c>
     </row>
     <row r="54" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A54" s="24" t="s">
+      <c r="A54" s="23" t="s">
         <v>68</v>
       </c>
-      <c r="B54" s="24" t="s">
+      <c r="B54" s="23" t="s">
         <v>120</v>
       </c>
       <c r="C54" s="12">
@@ -3072,10 +3460,10 @@
       </c>
     </row>
     <row r="55" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A55" s="24" t="s">
+      <c r="A55" s="23" t="s">
         <v>75</v>
       </c>
-      <c r="B55" s="24" t="s">
+      <c r="B55" s="23" t="s">
         <v>62</v>
       </c>
       <c r="C55" s="12">
@@ -3086,10 +3474,10 @@
       </c>
     </row>
     <row r="56" spans="1:4" ht="28.5" x14ac:dyDescent="0.25">
-      <c r="A56" s="24" t="s">
+      <c r="A56" s="23" t="s">
         <v>75</v>
       </c>
-      <c r="B56" s="24" t="s">
+      <c r="B56" s="23" t="s">
         <v>122</v>
       </c>
       <c r="C56" s="12">
@@ -3100,10 +3488,10 @@
       </c>
     </row>
     <row r="57" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A57" s="24" t="s">
+      <c r="A57" s="23" t="s">
         <v>75</v>
       </c>
-      <c r="B57" s="24" t="s">
+      <c r="B57" s="23" t="s">
         <v>120</v>
       </c>
       <c r="C57" s="12">
@@ -3114,10 +3502,10 @@
       </c>
     </row>
     <row r="58" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A58" s="24" t="s">
+      <c r="A58" s="23" t="s">
         <v>82</v>
       </c>
-      <c r="B58" s="24" t="s">
+      <c r="B58" s="23" t="s">
         <v>108</v>
       </c>
       <c r="C58" s="12">
@@ -3128,10 +3516,10 @@
       </c>
     </row>
     <row r="59" spans="1:4" ht="28.5" x14ac:dyDescent="0.25">
-      <c r="A59" s="24" t="s">
+      <c r="A59" s="23" t="s">
         <v>82</v>
       </c>
-      <c r="B59" s="24" t="s">
+      <c r="B59" s="23" t="s">
         <v>126</v>
       </c>
       <c r="C59" s="12">
@@ -3162,32 +3550,34 @@
     <col min="5" max="5" width="17.5703125" customWidth="1"/>
     <col min="6" max="6" width="22.85546875" customWidth="1"/>
     <col min="7" max="7" width="36.42578125" customWidth="1"/>
+    <col min="8" max="8" width="16.28515625" customWidth="1"/>
+    <col min="9" max="9" width="20.42578125" customWidth="1"/>
     <col min="10" max="10" width="23.85546875" customWidth="1"/>
     <col min="11" max="11" width="28.28515625" customWidth="1"/>
     <col min="12" max="12" width="38.140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" ht="16.5" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
       <c r="A1" s="10" t="s">
         <v>98</v>
       </c>
     </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
         <v>99</v>
       </c>
     </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
         <v>89</v>
       </c>
     </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" s="3" t="s">
         <v>90</v>
       </c>
     </row>
-    <row r="6" spans="1:8" ht="36" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:3" ht="36" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="15" t="s">
         <v>16</v>
       </c>
@@ -3198,173 +3588,127 @@
         <v>91</v>
       </c>
     </row>
-    <row r="7" spans="1:8" ht="36" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:3" ht="36" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="15" t="s">
         <v>92</v>
       </c>
       <c r="B7" s="16" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
       <c r="C7" s="17" t="s">
         <v>93</v>
       </c>
     </row>
-    <row r="8" spans="1:8" ht="36" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:3" ht="36" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="15" t="s">
         <v>94</v>
       </c>
       <c r="B8" s="16" t="s">
-        <v>142</v>
-      </c>
-    </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.25">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" s="3" t="s">
         <v>95</v>
       </c>
     </row>
-    <row r="14" spans="1:8" ht="45" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A14" s="11" t="s">
         <v>134</v>
       </c>
       <c r="B14" s="11" t="s">
         <v>23</v>
       </c>
-      <c r="C14" s="20" t="s">
-        <v>34</v>
-      </c>
-      <c r="D14" s="11" t="s">
-        <v>141</v>
-      </c>
-      <c r="G14" s="11" t="s">
-        <v>136</v>
-      </c>
-      <c r="H14" s="11" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="15" spans="1:8" ht="42.75" x14ac:dyDescent="0.25">
-      <c r="A15" s="23" t="s">
+      <c r="C14" s="11" t="s">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A15" s="22" t="s">
         <v>35</v>
       </c>
       <c r="B15" s="13">
         <v>46266</v>
       </c>
-      <c r="C15" s="21">
-        <v>1850000</v>
-      </c>
-      <c r="D15" s="25" t="s">
+      <c r="C15" s="24" t="s">
         <v>36</v>
       </c>
-      <c r="G15" s="23" t="s">
-        <v>107</v>
-      </c>
-      <c r="H15" s="12" t="s">
-        <v>106</v>
-      </c>
-    </row>
-    <row r="16" spans="1:8" ht="57" x14ac:dyDescent="0.25">
-      <c r="A16" s="23" t="s">
+    </row>
+    <row r="16" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A16" s="22" t="s">
         <v>35</v>
       </c>
       <c r="B16" s="13">
         <v>46266</v>
       </c>
-      <c r="C16" s="14">
-        <v>300000</v>
-      </c>
-      <c r="D16" s="25" t="s">
+      <c r="C16" s="24" t="s">
         <v>36</v>
       </c>
-      <c r="G16" s="23" t="s">
-        <v>110</v>
-      </c>
-      <c r="H16" s="12" t="s">
-        <v>111</v>
-      </c>
-    </row>
-    <row r="17" spans="1:12" ht="28.5" x14ac:dyDescent="0.25">
-      <c r="A17" s="23" t="s">
+    </row>
+    <row r="17" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A17" s="22" t="s">
         <v>46</v>
       </c>
       <c r="B17" s="13">
         <v>46275</v>
       </c>
-      <c r="C17" s="14">
-        <v>750000</v>
-      </c>
-      <c r="D17" s="25" t="s">
+      <c r="C17" s="24" t="s">
         <v>47</v>
       </c>
-      <c r="G17" s="23" t="s">
-        <v>64</v>
-      </c>
-      <c r="H17" s="12" t="s">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="18" spans="1:12" ht="28.5" x14ac:dyDescent="0.25">
-      <c r="A18" s="23" t="s">
+    </row>
+    <row r="18" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A18" s="22" t="s">
         <v>46</v>
       </c>
       <c r="B18" s="13">
         <v>46275</v>
       </c>
-      <c r="C18" s="14">
-        <v>150000</v>
-      </c>
-      <c r="D18" s="25" t="s">
+      <c r="C18" s="24" t="s">
         <v>47</v>
-      </c>
-      <c r="G18" s="23" t="s">
-        <v>118</v>
-      </c>
-      <c r="H18" s="12" t="s">
-        <v>119</v>
       </c>
       <c r="K18" s="12"/>
       <c r="L18" s="12"/>
     </row>
     <row r="19" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A19" s="23" t="s">
+      <c r="A19" s="22" t="s">
         <v>57</v>
       </c>
       <c r="B19" s="13">
         <v>46277</v>
       </c>
-      <c r="C19" s="14">
-        <v>1050000</v>
-      </c>
-      <c r="D19" s="25" t="s">
+      <c r="C19" s="24" t="s">
         <v>58</v>
       </c>
     </row>
     <row r="20" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A20" s="23" t="s">
+      <c r="A20" s="22" t="s">
         <v>68</v>
       </c>
       <c r="B20" s="13">
         <v>46280</v>
       </c>
-      <c r="C20" s="14">
-        <v>250000</v>
-      </c>
-      <c r="D20" s="25" t="s">
+      <c r="C20" s="24" t="s">
         <v>36</v>
+      </c>
+      <c r="G20" s="27" t="s">
+        <v>145</v>
       </c>
       <c r="K20" s="12"/>
       <c r="L20" s="12"/>
     </row>
-    <row r="21" spans="1:12" ht="45" x14ac:dyDescent="0.25">
-      <c r="A21" s="23" t="s">
+    <row r="21" spans="1:12" ht="30" x14ac:dyDescent="0.25">
+      <c r="A21" s="22" t="s">
         <v>68</v>
       </c>
       <c r="B21" s="13">
         <v>46280</v>
       </c>
-      <c r="C21" s="14">
-        <v>96000</v>
-      </c>
-      <c r="D21" s="25" t="s">
+      <c r="C21" s="24" t="s">
         <v>36</v>
       </c>
       <c r="G21" s="11" t="s">
@@ -3382,20 +3726,17 @@
       <c r="K21" s="12"/>
       <c r="L21" s="12"/>
     </row>
-    <row r="22" spans="1:12" ht="28.5" x14ac:dyDescent="0.25">
-      <c r="A22" s="23" t="s">
+    <row r="22" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A22" s="22" t="s">
         <v>75</v>
       </c>
       <c r="B22" s="13">
         <v>46283</v>
       </c>
-      <c r="C22" s="14">
-        <v>375000</v>
-      </c>
-      <c r="D22" s="25" t="s">
+      <c r="C22" s="24" t="s">
         <v>47</v>
       </c>
-      <c r="G22" s="23" t="s">
+      <c r="G22" s="22" t="s">
         <v>36</v>
       </c>
       <c r="H22" s="12" t="s">
@@ -3410,20 +3751,17 @@
       <c r="K22" s="12"/>
       <c r="L22" s="12"/>
     </row>
-    <row r="23" spans="1:12" ht="28.5" x14ac:dyDescent="0.25">
-      <c r="A23" s="23" t="s">
+    <row r="23" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A23" s="22" t="s">
         <v>75</v>
       </c>
       <c r="B23" s="13">
         <v>46283</v>
       </c>
-      <c r="C23" s="14">
-        <v>125000</v>
-      </c>
-      <c r="D23" s="25" t="s">
+      <c r="C23" s="24" t="s">
         <v>47</v>
       </c>
-      <c r="G23" s="23" t="s">
+      <c r="G23" s="22" t="s">
         <v>47</v>
       </c>
       <c r="H23" s="12" t="s">
@@ -3438,20 +3776,17 @@
       <c r="K23" s="12"/>
       <c r="L23" s="12"/>
     </row>
-    <row r="24" spans="1:12" ht="28.5" x14ac:dyDescent="0.25">
-      <c r="A24" s="23" t="s">
+    <row r="24" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A24" s="22" t="s">
         <v>75</v>
       </c>
       <c r="B24" s="13">
         <v>46283</v>
       </c>
-      <c r="C24" s="14">
-        <v>48000</v>
-      </c>
-      <c r="D24" s="25" t="s">
+      <c r="C24" s="24" t="s">
         <v>47</v>
       </c>
-      <c r="G24" s="23" t="s">
+      <c r="G24" s="22" t="s">
         <v>58</v>
       </c>
       <c r="H24" s="12" t="s">
@@ -3467,16 +3802,13 @@
       <c r="L24" s="12"/>
     </row>
     <row r="25" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A25" s="23" t="s">
+      <c r="A25" s="22" t="s">
         <v>82</v>
       </c>
       <c r="B25" s="13">
         <v>46285</v>
       </c>
-      <c r="C25" s="14">
-        <v>3700000</v>
-      </c>
-      <c r="D25" s="25" t="s">
+      <c r="C25" s="24" t="s">
         <v>58</v>
       </c>
       <c r="H25" s="12"/>
@@ -3485,25 +3817,55 @@
       <c r="L25" s="12"/>
     </row>
     <row r="26" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A26" s="23" t="s">
+      <c r="A26" s="22" t="s">
         <v>82</v>
       </c>
       <c r="B26" s="13">
         <v>46285</v>
       </c>
-      <c r="C26" s="14">
-        <v>750000</v>
-      </c>
-      <c r="D26" s="25" t="s">
+      <c r="C26" s="24" t="s">
         <v>58</v>
       </c>
       <c r="F26" s="12"/>
-      <c r="G26" s="12"/>
+      <c r="G26" s="12" t="s">
+        <v>250</v>
+      </c>
       <c r="I26" s="12"/>
       <c r="J26" s="12"/>
       <c r="K26" s="12"/>
       <c r="L26" s="12"/>
     </row>
+    <row r="27" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="G27" s="11" t="s">
+        <v>136</v>
+      </c>
+      <c r="H27" s="11" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="28" spans="1:12" ht="28.5" x14ac:dyDescent="0.25">
+      <c r="G28" s="22" t="s">
+        <v>107</v>
+      </c>
+      <c r="H28" s="12" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="29" spans="1:12" ht="28.5" x14ac:dyDescent="0.25">
+      <c r="G29" s="22" t="s">
+        <v>110</v>
+      </c>
+      <c r="H29" s="12" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="30" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A30" t="s">
+        <v>252</v>
+      </c>
+      <c r="G30" s="22"/>
+      <c r="H30" s="12"/>
+    </row>
     <row r="31" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A31" s="11" t="s">
         <v>137</v>
@@ -3512,122 +3874,158 @@
         <v>29</v>
       </c>
       <c r="C31" s="11" t="s">
-        <v>140</v>
+        <v>33</v>
+      </c>
+      <c r="D31" s="11" t="s">
+        <v>138</v>
+      </c>
+      <c r="G31" s="22" t="s">
+        <v>118</v>
+      </c>
+      <c r="H31" s="12" t="s">
+        <v>119</v>
       </c>
     </row>
     <row r="32" spans="1:12" ht="28.5" x14ac:dyDescent="0.25">
-      <c r="A32" s="23" t="s">
+      <c r="A32" s="22" t="s">
         <v>108</v>
       </c>
       <c r="B32" s="12" t="s">
         <v>113</v>
       </c>
-      <c r="C32" s="25" t="s">
+      <c r="C32" s="19" t="s">
+        <v>127</v>
+      </c>
+      <c r="D32" s="24" t="s">
         <v>107</v>
       </c>
     </row>
     <row r="33" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A33" s="23" t="s">
+      <c r="A33" s="22" t="s">
         <v>109</v>
       </c>
       <c r="B33" s="12" t="s">
         <v>112</v>
       </c>
-      <c r="C33" s="25" t="s">
+      <c r="C33" s="14">
+        <v>150000</v>
+      </c>
+      <c r="D33" s="24" t="s">
         <v>110</v>
       </c>
     </row>
     <row r="34" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A34" s="23" t="s">
+      <c r="A34" s="22" t="s">
         <v>115</v>
       </c>
       <c r="B34" s="12" t="s">
         <v>114</v>
       </c>
-      <c r="C34" s="25" t="s">
+      <c r="C34" s="14">
+        <v>750000</v>
+      </c>
+      <c r="D34" s="24" t="s">
         <v>64</v>
       </c>
     </row>
     <row r="35" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A35" s="23" t="s">
+      <c r="A35" s="22" t="s">
         <v>62</v>
       </c>
       <c r="B35" s="12" t="s">
         <v>63</v>
       </c>
-      <c r="C35" s="25" t="s">
+      <c r="C35" s="14">
+        <v>150000</v>
+      </c>
+      <c r="D35" s="24" t="s">
         <v>64</v>
       </c>
     </row>
     <row r="36" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A36" s="23" t="s">
+      <c r="A36" s="22" t="s">
         <v>116</v>
       </c>
       <c r="B36" s="12" t="s">
         <v>117</v>
       </c>
-      <c r="C36" s="26" t="s">
+      <c r="C36" s="14">
+        <v>350000</v>
+      </c>
+      <c r="D36" s="25" t="s">
         <v>118</v>
       </c>
     </row>
     <row r="37" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A37" s="23" t="s">
+      <c r="A37" s="22" t="s">
         <v>120</v>
       </c>
       <c r="B37" s="12" t="s">
         <v>121</v>
       </c>
-      <c r="C37" s="26" t="s">
+      <c r="C37" s="14">
+        <v>25000</v>
+      </c>
+      <c r="D37" s="25" t="s">
         <v>118</v>
       </c>
+    </row>
+    <row r="38" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D38" s="14"/>
+    </row>
+    <row r="39" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A39" s="27" t="s">
+        <v>251</v>
+      </c>
+      <c r="D39" s="14"/>
     </row>
     <row r="40" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A40" s="11" t="s">
-        <v>138</v>
+        <v>142</v>
       </c>
       <c r="B40" s="11" t="s">
-        <v>139</v>
+        <v>143</v>
       </c>
       <c r="C40" s="11" t="s">
         <v>32</v>
       </c>
-      <c r="D40" s="11" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="41" spans="1:4" ht="28.5" x14ac:dyDescent="0.25">
-      <c r="A41" s="24" t="s">
+      <c r="D40" s="20" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="41" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A41" s="23" t="s">
         <v>35</v>
       </c>
-      <c r="B41" s="24" t="s">
+      <c r="B41" s="23" t="s">
         <v>108</v>
       </c>
       <c r="C41" s="19">
         <v>1</v>
       </c>
-      <c r="D41" s="19" t="s">
-        <v>127</v>
+      <c r="D41" s="21">
+        <v>1850000</v>
       </c>
     </row>
     <row r="42" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A42" s="24" t="s">
+      <c r="A42" s="23" t="s">
         <v>35</v>
       </c>
-      <c r="B42" s="24" t="s">
+      <c r="B42" s="23" t="s">
         <v>109</v>
       </c>
       <c r="C42" s="12">
         <v>2</v>
       </c>
       <c r="D42" s="14">
-        <v>150000</v>
+        <v>300000</v>
       </c>
     </row>
     <row r="43" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A43" s="24" t="s">
+      <c r="A43" s="23" t="s">
         <v>46</v>
       </c>
-      <c r="B43" s="24" t="s">
+      <c r="B43" s="23" t="s">
         <v>115</v>
       </c>
       <c r="C43" s="12">
@@ -3638,10 +4036,10 @@
       </c>
     </row>
     <row r="44" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A44" s="24" t="s">
+      <c r="A44" s="23" t="s">
         <v>46</v>
       </c>
-      <c r="B44" s="24" t="s">
+      <c r="B44" s="23" t="s">
         <v>109</v>
       </c>
       <c r="C44" s="12">
@@ -3652,52 +4050,52 @@
       </c>
     </row>
     <row r="45" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A45" s="24" t="s">
+      <c r="A45" s="23" t="s">
         <v>57</v>
       </c>
-      <c r="B45" s="24" t="s">
+      <c r="B45" s="23" t="s">
         <v>62</v>
       </c>
       <c r="C45" s="12">
         <v>3</v>
       </c>
       <c r="D45" s="14">
-        <v>350000</v>
+        <v>1050000</v>
       </c>
     </row>
     <row r="46" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A46" s="24" t="s">
+      <c r="A46" s="23" t="s">
         <v>68</v>
       </c>
-      <c r="B46" s="24" t="s">
+      <c r="B46" s="23" t="s">
         <v>116</v>
       </c>
       <c r="C46" s="12">
         <v>10</v>
       </c>
       <c r="D46" s="14">
-        <v>25000</v>
+        <v>250000</v>
       </c>
     </row>
     <row r="47" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A47" s="24" t="s">
+      <c r="A47" s="23" t="s">
         <v>68</v>
       </c>
-      <c r="B47" s="24" t="s">
+      <c r="B47" s="23" t="s">
         <v>120</v>
       </c>
       <c r="C47" s="12">
         <v>2</v>
       </c>
       <c r="D47" s="14">
-        <v>48000</v>
+        <v>96000</v>
       </c>
     </row>
     <row r="48" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A48" s="24" t="s">
+      <c r="A48" s="23" t="s">
         <v>75</v>
       </c>
-      <c r="B48" s="24" t="s">
+      <c r="B48" s="23" t="s">
         <v>62</v>
       </c>
       <c r="C48" s="12">
@@ -3708,24 +4106,24 @@
       </c>
     </row>
     <row r="49" spans="1:4" ht="28.5" x14ac:dyDescent="0.25">
-      <c r="A49" s="24" t="s">
+      <c r="A49" s="23" t="s">
         <v>75</v>
       </c>
-      <c r="B49" s="24" t="s">
+      <c r="B49" s="23" t="s">
         <v>122</v>
       </c>
       <c r="C49" s="12">
         <v>5</v>
       </c>
       <c r="D49" s="14">
-        <v>25000</v>
+        <v>125000</v>
       </c>
     </row>
     <row r="50" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A50" s="24" t="s">
+      <c r="A50" s="23" t="s">
         <v>75</v>
       </c>
-      <c r="B50" s="24" t="s">
+      <c r="B50" s="23" t="s">
         <v>120</v>
       </c>
       <c r="C50" s="12">
@@ -3736,24 +4134,24 @@
       </c>
     </row>
     <row r="51" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A51" s="24" t="s">
+      <c r="A51" s="23" t="s">
         <v>82</v>
       </c>
-      <c r="B51" s="24" t="s">
+      <c r="B51" s="23" t="s">
         <v>108</v>
       </c>
       <c r="C51" s="12">
         <v>2</v>
       </c>
       <c r="D51" s="14">
-        <v>1850000</v>
+        <v>3700000</v>
       </c>
     </row>
     <row r="52" spans="1:4" ht="28.5" x14ac:dyDescent="0.25">
-      <c r="A52" s="24" t="s">
+      <c r="A52" s="23" t="s">
         <v>82</v>
       </c>
-      <c r="B52" s="24" t="s">
+      <c r="B52" s="23" t="s">
         <v>126</v>
       </c>
       <c r="C52" s="12">
@@ -3770,6 +4168,618 @@
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0DA06C20-0B0B-43BE-81EE-9BBEACE60F15}">
+  <dimension ref="A1:B139"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData>
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="B6" t="s">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="15" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="16" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="17" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="18" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
+        <v>157</v>
+      </c>
+    </row>
+    <row r="19" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A19" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="20" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A20" t="s">
+        <v>159</v>
+      </c>
+    </row>
+    <row r="23" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A23" t="s">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="24" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A24" t="s">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="25" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A25" t="s">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="27" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A27" t="s">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="28" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A28" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="29" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A29" t="s">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="30" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A30" t="s">
+        <v>166</v>
+      </c>
+    </row>
+    <row r="31" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A31" t="s">
+        <v>159</v>
+      </c>
+    </row>
+    <row r="33" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A33" t="s">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="34" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A34" t="s">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="35" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A35" t="s">
+        <v>169</v>
+      </c>
+    </row>
+    <row r="36" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A36" t="s">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="37" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A37" t="s">
+        <v>159</v>
+      </c>
+    </row>
+    <row r="40" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A40" t="s">
+        <v>171</v>
+      </c>
+    </row>
+    <row r="41" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A41" t="s">
+        <v>172</v>
+      </c>
+    </row>
+    <row r="42" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A42" t="s">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="43" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A43" t="s">
+        <v>174</v>
+      </c>
+    </row>
+    <row r="44" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A44" t="s">
+        <v>175</v>
+      </c>
+    </row>
+    <row r="45" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A45" t="s">
+        <v>176</v>
+      </c>
+    </row>
+    <row r="46" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A46" t="s">
+        <v>159</v>
+      </c>
+    </row>
+    <row r="49" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A49" t="s">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="50" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A50" t="s">
+        <v>178</v>
+      </c>
+    </row>
+    <row r="51" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A51" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="52" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A52" t="s">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="53" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A53" t="s">
+        <v>181</v>
+      </c>
+    </row>
+    <row r="55" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A55" t="s">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="56" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A56" t="s">
+        <v>159</v>
+      </c>
+    </row>
+    <row r="57" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A57" t="s">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="59" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A59" t="s">
+        <v>183</v>
+      </c>
+    </row>
+    <row r="60" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A60" t="s">
+        <v>184</v>
+      </c>
+    </row>
+    <row r="61" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A61" t="s">
+        <v>185</v>
+      </c>
+    </row>
+    <row r="62" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A62" t="s">
+        <v>186</v>
+      </c>
+    </row>
+    <row r="63" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A63" t="s">
+        <v>187</v>
+      </c>
+    </row>
+    <row r="65" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A65" t="s">
+        <v>188</v>
+      </c>
+    </row>
+    <row r="66" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A66" t="s">
+        <v>189</v>
+      </c>
+    </row>
+    <row r="67" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A67" t="s">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="68" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A68" t="s">
+        <v>186</v>
+      </c>
+    </row>
+    <row r="69" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A69" t="s">
+        <v>187</v>
+      </c>
+    </row>
+    <row r="70" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A70" t="s">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="72" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A72" t="s">
+        <v>191</v>
+      </c>
+    </row>
+    <row r="73" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A73" t="s">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="74" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A74" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="75" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A75" t="s">
+        <v>186</v>
+      </c>
+    </row>
+    <row r="76" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A76" t="s">
+        <v>187</v>
+      </c>
+    </row>
+    <row r="77" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A77" t="s">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="79" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A79" t="s">
+        <v>194</v>
+      </c>
+    </row>
+    <row r="80" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A80" t="s">
+        <v>195</v>
+      </c>
+    </row>
+    <row r="81" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A81" t="s">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="82" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A82" t="s">
+        <v>197</v>
+      </c>
+    </row>
+    <row r="83" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A83" t="s">
+        <v>186</v>
+      </c>
+    </row>
+    <row r="84" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A84" t="s">
+        <v>187</v>
+      </c>
+    </row>
+    <row r="85" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A85" t="s">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="87" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A87" t="s">
+        <v>198</v>
+      </c>
+    </row>
+    <row r="88" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A88" t="s">
+        <v>199</v>
+      </c>
+    </row>
+    <row r="89" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A89" t="s">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="90" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A90" t="s">
+        <v>201</v>
+      </c>
+    </row>
+    <row r="92" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A92" t="s">
+        <v>202</v>
+      </c>
+    </row>
+    <row r="93" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A93" t="s">
+        <v>203</v>
+      </c>
+    </row>
+    <row r="94" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A94" t="s">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="95" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A95" t="s">
+        <v>205</v>
+      </c>
+    </row>
+    <row r="96" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A96" t="s">
+        <v>206</v>
+      </c>
+    </row>
+    <row r="97" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A97" t="s">
+        <v>207</v>
+      </c>
+    </row>
+    <row r="98" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A98" t="s">
+        <v>208</v>
+      </c>
+    </row>
+    <row r="100" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A100" t="s">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="101" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A101" t="s">
+        <v>210</v>
+      </c>
+      <c r="B101" t="s">
+        <v>211</v>
+      </c>
+    </row>
+    <row r="102" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A102" t="s">
+        <v>212</v>
+      </c>
+      <c r="B102" t="s">
+        <v>213</v>
+      </c>
+    </row>
+    <row r="103" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A103" t="s">
+        <v>214</v>
+      </c>
+      <c r="B103" t="s">
+        <v>215</v>
+      </c>
+    </row>
+    <row r="105" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A105" t="s">
+        <v>216</v>
+      </c>
+    </row>
+    <row r="106" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A106" t="s">
+        <v>217</v>
+      </c>
+      <c r="B106" t="s">
+        <v>218</v>
+      </c>
+    </row>
+    <row r="107" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A107" t="s">
+        <v>219</v>
+      </c>
+      <c r="B107" t="s">
+        <v>220</v>
+      </c>
+    </row>
+    <row r="108" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A108" t="s">
+        <v>221</v>
+      </c>
+      <c r="B108" t="s">
+        <v>222</v>
+      </c>
+    </row>
+    <row r="109" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A109" t="s">
+        <v>223</v>
+      </c>
+      <c r="B109" t="s">
+        <v>218</v>
+      </c>
+    </row>
+    <row r="110" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A110" t="s">
+        <v>224</v>
+      </c>
+      <c r="B110" t="s">
+        <v>220</v>
+      </c>
+    </row>
+    <row r="111" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A111" t="s">
+        <v>225</v>
+      </c>
+      <c r="B111" t="s">
+        <v>226</v>
+      </c>
+    </row>
+    <row r="114" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A114" t="s">
+        <v>227</v>
+      </c>
+    </row>
+    <row r="115" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A115" t="s">
+        <v>228</v>
+      </c>
+    </row>
+    <row r="116" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A116" t="s">
+        <v>229</v>
+      </c>
+    </row>
+    <row r="117" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A117" t="s">
+        <v>230</v>
+      </c>
+    </row>
+    <row r="118" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A118" t="s">
+        <v>231</v>
+      </c>
+    </row>
+    <row r="119" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A119" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="120" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A120" t="s">
+        <v>233</v>
+      </c>
+    </row>
+    <row r="121" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A121" t="s">
+        <v>234</v>
+      </c>
+    </row>
+    <row r="122" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A122" t="s">
+        <v>235</v>
+      </c>
+    </row>
+    <row r="123" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A123" t="s">
+        <v>236</v>
+      </c>
+    </row>
+    <row r="124" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A124" t="s">
+        <v>237</v>
+      </c>
+    </row>
+    <row r="125" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A125" t="s">
+        <v>238</v>
+      </c>
+    </row>
+    <row r="126" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A126" t="s">
+        <v>239</v>
+      </c>
+    </row>
+    <row r="129" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A129" t="s">
+        <v>240</v>
+      </c>
+    </row>
+    <row r="130" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A130" t="s">
+        <v>241</v>
+      </c>
+    </row>
+    <row r="131" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A131" t="s">
+        <v>242</v>
+      </c>
+    </row>
+    <row r="132" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A132" t="s">
+        <v>243</v>
+      </c>
+    </row>
+    <row r="133" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A133" t="s">
+        <v>244</v>
+      </c>
+    </row>
+    <row r="135" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A135" t="s">
+        <v>245</v>
+      </c>
+    </row>
+    <row r="136" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A136" t="s">
+        <v>246</v>
+      </c>
+    </row>
+    <row r="137" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A137" t="s">
+        <v>247</v>
+      </c>
+    </row>
+    <row r="138" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A138" t="s">
+        <v>248</v>
+      </c>
+    </row>
+    <row r="139" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A139" t="s">
+        <v>249</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6DC48F45-D148-4F30-9580-FDB05BB3978E}">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{545EEB48-EB00-4A4C-BE0D-21AE85A0FA9D}">
   <dimension ref="A2:R73"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -4199,7 +5209,7 @@
       </c>
     </row>
     <row r="29" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A29" s="24" t="s">
+      <c r="A29" s="23" t="s">
         <v>35</v>
       </c>
       <c r="B29" s="13">
@@ -4222,7 +5232,7 @@
       </c>
     </row>
     <row r="30" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A30" s="24" t="s">
+      <c r="A30" s="23" t="s">
         <v>35</v>
       </c>
       <c r="B30" s="13">
@@ -4245,7 +5255,7 @@
       </c>
     </row>
     <row r="31" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A31" s="24" t="s">
+      <c r="A31" s="23" t="s">
         <v>46</v>
       </c>
       <c r="B31" s="13">
@@ -4268,7 +5278,7 @@
       </c>
     </row>
     <row r="32" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A32" s="24" t="s">
+      <c r="A32" s="23" t="s">
         <v>46</v>
       </c>
       <c r="B32" s="13">
@@ -4291,7 +5301,7 @@
       </c>
     </row>
     <row r="33" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A33" s="24" t="s">
+      <c r="A33" s="23" t="s">
         <v>57</v>
       </c>
       <c r="B33" s="13">
@@ -4314,7 +5324,7 @@
       </c>
     </row>
     <row r="34" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A34" s="24" t="s">
+      <c r="A34" s="23" t="s">
         <v>68</v>
       </c>
       <c r="B34" s="13">
@@ -4337,7 +5347,7 @@
       </c>
     </row>
     <row r="35" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A35" s="24" t="s">
+      <c r="A35" s="23" t="s">
         <v>68</v>
       </c>
       <c r="B35" s="13">
@@ -4360,7 +5370,7 @@
       </c>
     </row>
     <row r="36" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A36" s="24" t="s">
+      <c r="A36" s="23" t="s">
         <v>75</v>
       </c>
       <c r="B36" s="13">
@@ -4383,7 +5393,7 @@
       </c>
     </row>
     <row r="37" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A37" s="24" t="s">
+      <c r="A37" s="23" t="s">
         <v>75</v>
       </c>
       <c r="B37" s="13">
@@ -4406,7 +5416,7 @@
       </c>
     </row>
     <row r="38" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A38" s="24" t="s">
+      <c r="A38" s="23" t="s">
         <v>75</v>
       </c>
       <c r="B38" s="13">
@@ -4429,7 +5439,7 @@
       </c>
     </row>
     <row r="39" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A39" s="24" t="s">
+      <c r="A39" s="23" t="s">
         <v>82</v>
       </c>
       <c r="B39" s="13">
@@ -4452,7 +5462,7 @@
       </c>
     </row>
     <row r="40" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A40" s="24" t="s">
+      <c r="A40" s="23" t="s">
         <v>82</v>
       </c>
       <c r="B40" s="13">
@@ -4489,7 +5499,7 @@
       </c>
     </row>
     <row r="46" spans="1:7" ht="28.5" x14ac:dyDescent="0.25">
-      <c r="A46" s="24" t="s">
+      <c r="A46" s="23" t="s">
         <v>108</v>
       </c>
       <c r="B46" s="12" t="s">
@@ -4503,7 +5513,7 @@
       </c>
     </row>
     <row r="47" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A47" s="24" t="s">
+      <c r="A47" s="23" t="s">
         <v>109</v>
       </c>
       <c r="B47" s="12" t="s">
@@ -4517,7 +5527,7 @@
       </c>
     </row>
     <row r="48" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A48" s="24" t="s">
+      <c r="A48" s="23" t="s">
         <v>115</v>
       </c>
       <c r="B48" s="12" t="s">
@@ -4531,7 +5541,7 @@
       </c>
     </row>
     <row r="49" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A49" s="24" t="s">
+      <c r="A49" s="23" t="s">
         <v>109</v>
       </c>
       <c r="B49" s="12" t="s">
@@ -4545,7 +5555,7 @@
       </c>
     </row>
     <row r="50" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A50" s="24" t="s">
+      <c r="A50" s="23" t="s">
         <v>62</v>
       </c>
       <c r="B50" s="12" t="s">
@@ -4559,7 +5569,7 @@
       </c>
     </row>
     <row r="51" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A51" s="24" t="s">
+      <c r="A51" s="23" t="s">
         <v>116</v>
       </c>
       <c r="B51" s="12" t="s">
@@ -4573,7 +5583,7 @@
       </c>
     </row>
     <row r="52" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A52" s="24" t="s">
+      <c r="A52" s="23" t="s">
         <v>120</v>
       </c>
       <c r="B52" s="12" t="s">
@@ -4587,7 +5597,7 @@
       </c>
     </row>
     <row r="53" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A53" s="24" t="s">
+      <c r="A53" s="23" t="s">
         <v>62</v>
       </c>
       <c r="B53" s="12" t="s">
@@ -4601,7 +5611,7 @@
       </c>
     </row>
     <row r="54" spans="1:4" ht="28.5" x14ac:dyDescent="0.25">
-      <c r="A54" s="24" t="s">
+      <c r="A54" s="23" t="s">
         <v>122</v>
       </c>
       <c r="B54" s="12" t="s">
@@ -4615,7 +5625,7 @@
       </c>
     </row>
     <row r="55" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A55" s="24" t="s">
+      <c r="A55" s="23" t="s">
         <v>120</v>
       </c>
       <c r="B55" s="12" t="s">
@@ -4629,7 +5639,7 @@
       </c>
     </row>
     <row r="56" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A56" s="24" t="s">
+      <c r="A56" s="23" t="s">
         <v>108</v>
       </c>
       <c r="B56" s="12" t="s">
@@ -4643,7 +5653,7 @@
       </c>
     </row>
     <row r="57" spans="1:4" ht="28.5" x14ac:dyDescent="0.25">
-      <c r="A57" s="24" t="s">
+      <c r="A57" s="23" t="s">
         <v>126</v>
       </c>
       <c r="B57" s="12" t="s">
@@ -4671,10 +5681,10 @@
       </c>
     </row>
     <row r="62" spans="1:4" ht="28.5" x14ac:dyDescent="0.25">
-      <c r="A62" s="24" t="s">
+      <c r="A62" s="23" t="s">
         <v>35</v>
       </c>
-      <c r="B62" s="24" t="s">
+      <c r="B62" s="23" t="s">
         <v>108</v>
       </c>
       <c r="C62" s="19">
@@ -4685,10 +5695,10 @@
       </c>
     </row>
     <row r="63" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A63" s="24" t="s">
+      <c r="A63" s="23" t="s">
         <v>35</v>
       </c>
-      <c r="B63" s="24" t="s">
+      <c r="B63" s="23" t="s">
         <v>109</v>
       </c>
       <c r="C63" s="12">
@@ -4699,10 +5709,10 @@
       </c>
     </row>
     <row r="64" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A64" s="24" t="s">
+      <c r="A64" s="23" t="s">
         <v>46</v>
       </c>
-      <c r="B64" s="24" t="s">
+      <c r="B64" s="23" t="s">
         <v>115</v>
       </c>
       <c r="C64" s="12">
@@ -4713,10 +5723,10 @@
       </c>
     </row>
     <row r="65" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A65" s="24" t="s">
+      <c r="A65" s="23" t="s">
         <v>46</v>
       </c>
-      <c r="B65" s="24" t="s">
+      <c r="B65" s="23" t="s">
         <v>109</v>
       </c>
       <c r="C65" s="12">
@@ -4727,10 +5737,10 @@
       </c>
     </row>
     <row r="66" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A66" s="24" t="s">
+      <c r="A66" s="23" t="s">
         <v>57</v>
       </c>
-      <c r="B66" s="24" t="s">
+      <c r="B66" s="23" t="s">
         <v>62</v>
       </c>
       <c r="C66" s="12">
@@ -4741,10 +5751,10 @@
       </c>
     </row>
     <row r="67" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A67" s="24" t="s">
+      <c r="A67" s="23" t="s">
         <v>68</v>
       </c>
-      <c r="B67" s="24" t="s">
+      <c r="B67" s="23" t="s">
         <v>116</v>
       </c>
       <c r="C67" s="12">
@@ -4755,10 +5765,10 @@
       </c>
     </row>
     <row r="68" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A68" s="24" t="s">
+      <c r="A68" s="23" t="s">
         <v>68</v>
       </c>
-      <c r="B68" s="24" t="s">
+      <c r="B68" s="23" t="s">
         <v>120</v>
       </c>
       <c r="C68" s="12">
@@ -4769,10 +5779,10 @@
       </c>
     </row>
     <row r="69" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A69" s="24" t="s">
+      <c r="A69" s="23" t="s">
         <v>75</v>
       </c>
-      <c r="B69" s="24" t="s">
+      <c r="B69" s="23" t="s">
         <v>62</v>
       </c>
       <c r="C69" s="12">
@@ -4783,10 +5793,10 @@
       </c>
     </row>
     <row r="70" spans="1:4" ht="28.5" x14ac:dyDescent="0.25">
-      <c r="A70" s="24" t="s">
+      <c r="A70" s="23" t="s">
         <v>75</v>
       </c>
-      <c r="B70" s="24" t="s">
+      <c r="B70" s="23" t="s">
         <v>122</v>
       </c>
       <c r="C70" s="12">
@@ -4797,10 +5807,10 @@
       </c>
     </row>
     <row r="71" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A71" s="24" t="s">
+      <c r="A71" s="23" t="s">
         <v>75</v>
       </c>
-      <c r="B71" s="24" t="s">
+      <c r="B71" s="23" t="s">
         <v>120</v>
       </c>
       <c r="C71" s="12">
@@ -4811,10 +5821,10 @@
       </c>
     </row>
     <row r="72" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A72" s="24" t="s">
+      <c r="A72" s="23" t="s">
         <v>82</v>
       </c>
-      <c r="B72" s="24" t="s">
+      <c r="B72" s="23" t="s">
         <v>108</v>
       </c>
       <c r="C72" s="12">
@@ -4825,10 +5835,10 @@
       </c>
     </row>
     <row r="73" spans="1:4" ht="28.5" x14ac:dyDescent="0.25">
-      <c r="A73" s="24" t="s">
+      <c r="A73" s="23" t="s">
         <v>82</v>
       </c>
-      <c r="B73" s="24" t="s">
+      <c r="B73" s="23" t="s">
         <v>126</v>
       </c>
       <c r="C73" s="12">

</xml_diff>